<commit_message>
add the multi agent variant behind a flag
</commit_message>
<xml_diff>
--- a/data/sample.xlsx
+++ b/data/sample.xlsx
@@ -897,6 +897,88 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Units by Product</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Sheet1'!D1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Sheet1'!$B$2:$B$16</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Sheet1'!$D$2:$D$16</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -982,6 +1064,28 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>64</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="5" name="Chart 5"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId5"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1306,7 +1410,11 @@
           <t>Notes</t>
         </is>
       </c>
-      <c r="I1" s="2" t="n"/>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Profit</t>
+        </is>
+      </c>
       <c r="J1" s="2" t="n"/>
       <c r="K1" s="2" t="n"/>
       <c r="L1" s="2" t="n"/>
@@ -1338,8 +1446,14 @@
       <c r="G2" s="3" t="n">
         <v>46036</v>
       </c>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="n"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>top region</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>100</v>
+      </c>
       <c r="J2" s="2" t="n"/>
       <c r="K2" s="2" t="n"/>
       <c r="L2" s="2" t="n"/>
@@ -1376,7 +1490,9 @@
           <t>bulk order</t>
         </is>
       </c>
-      <c r="I3" s="2" t="n"/>
+      <c r="I3" s="2" t="n">
+        <v>200</v>
+      </c>
       <c r="J3" s="2" t="n"/>
       <c r="K3" s="2" t="n"/>
       <c r="L3" s="2" t="n"/>

</xml_diff>

<commit_message>
separate local/sheet prompts + untangle registry.py from local tools
</commit_message>
<xml_diff>
--- a/data/sample.xlsx
+++ b/data/sample.xlsx
@@ -979,6 +979,88 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Profit by Product</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Sheet1'!I1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Sheet1'!$B$2:$B$15</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Sheet1'!$I$2:$I$15</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -1086,6 +1168,28 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId5"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>80</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="6" name="Chart 6"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId6"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>

</xml_diff>